<commit_message>
progress: 46 village workbooks (rw-rtx-3070 2026-10-09T23:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Karani_13.334976_80.052422.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Karani_13.334976_80.052422.xlsx
@@ -1358,6 +1358,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1365,6 +1370,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 4, 5A, 5B, 6A, 6B, 6C, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1372,6 +1382,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12A, 12B, 13, 14, 15A, 15B, 16, 17A, 17B, 1A, 1B, 1C, 2, 3, 4, 5A, 5B, 5C, 5D, 6, 7A, 7B, 7C, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1379,6 +1394,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16A1, 16A2, 16A3, 16B1, 16B2, 17, 2, 3, 4A, 4B, 5, 6A, 6B, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1386,6 +1406,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A1A1, 16A2, 16B, 17, 18A1, 18B, 18C, 18D, 19A, 2, 20A, 20B, 21A, 21B1A, 21B2, 21B3, 22, 23A1, 23A2, 23B, 24A, 24B, 24C, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1393,6 +1418,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 2, 3, 4A1, 4A2, 4B1A1A, 4B1B, 4B1C, 4B1D, 4B2A, 4B2B, 5A, 5B, 5C1, 5C2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1400,6 +1430,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10C, 11, 12, 13A, 13B, 13C, 14, 15, 16, 2, 3A1A, 3A1B, 3A1C, 3A2, 3B1A, 3B1B, 3B2, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1407,11 +1442,21 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
           <t>9</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>